<commit_message>
Fix 2 sentence length.
</commit_message>
<xml_diff>
--- a/data/paragraph_hate_speech.xlsx
+++ b/data/paragraph_hate_speech.xlsx
@@ -6328,12 +6328,12 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>jel to onaj momak sto je degeneka slao po cevape kod "junuza",haa cigani??? Da to je bilo onda kada ste svi u paketu isli kod Jonuza na cevape na -30</t>
+          <t>jel to onaj momak sto je degeneka slao po cevape kod "junuza". haa cigani??? Da to je bilo onda kada ste svi u paketu isli kod Jonuza na cevape na -30</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>1b,1b</t>
+          <t>1b,1b,1b</t>
         </is>
       </c>
     </row>

</xml_diff>